<commit_message>
Insurgentes SD: split beams match the model tramos (EJE-5 S1, T-5 S3, T-6 S2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mu9wxeehZ5MxBaqNG8frbT
</commit_message>
<xml_diff>
--- a/revit/ArmadoTrabes_Insurgentes/Correccion_Roof_Garden_N10.xlsx
+++ b/revit/ArmadoTrabes_Insurgentes/Correccion_Roof_Garden_N10.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S34"/>
+  <dimension ref="A1:S28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -779,38 +779,38 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EJE-5 [S1]</t>
+          <t>EJE-5 [S2]</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>1 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>CS1 (cambio de sección)</t>
+          <t>2 (muro)</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.63</v>
+        <v>1.63</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>20x80</t>
+          <t>15x60</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>3#8</t>
+          <t>3#4</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>3#8</t>
+          <t>3#4</t>
         </is>
       </c>
       <c r="J5" s="2" t="n"/>
@@ -830,7 +830,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S5" s="2" t="n"/>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas: 15X80 ejes N-L (S1, incluye la pieza de 20x80) y 15X60 ejes K-B (S2).</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -840,38 +844,38 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>EJE-5 [S1]</t>
+          <t>EJE-5 [S2]</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>CS1 (cambio de sección)</t>
+          <t>2 (muro)</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>5 (muro bajo la viga)</t>
+          <t>3 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.63</v>
+        <v>1.81</v>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>20x80</t>
+          <t>15x60</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>3#8</t>
+          <t>3#4</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>3#8</t>
+          <t>3#4</t>
         </is>
       </c>
       <c r="J6" s="2" t="n"/>
@@ -905,20 +909,20 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>1 (muro bajo la viga)</t>
+          <t>3 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>2 (muro)</t>
+          <t>4 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1.63</v>
+        <v>1.81</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
@@ -936,9 +940,17 @@
         </is>
       </c>
       <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>2#4 60/60</t>
+        </is>
+      </c>
       <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>2#4 60/60</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="n"/>
       <c r="P7" s="2" t="inlineStr">
@@ -952,11 +964,7 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S7" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas: 15X80 ejes N-L (S1, incluye la pieza de 20x80) y 15X60 ejes K-B (S2).</t>
-        </is>
-      </c>
+      <c r="S7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -970,20 +978,20 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>2 (muro)</t>
+          <t>4 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>3 (muro bajo la viga)</t>
+          <t>5 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1.81</v>
+        <v>1.83</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
@@ -1031,20 +1039,20 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>3 (muro bajo la viga)</t>
+          <t>5 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>4 (muro bajo la viga)</t>
+          <t>6 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1.81</v>
+        <v>1.72</v>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
@@ -1062,17 +1070,9 @@
         </is>
       </c>
       <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2#4 60/60</t>
-        </is>
-      </c>
+      <c r="K9" s="2" t="n"/>
       <c r="L9" s="2" t="n"/>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>2#4 60/60</t>
-        </is>
-      </c>
+      <c r="M9" s="2" t="n"/>
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="inlineStr">
@@ -1100,16 +1100,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>4 (muro bajo la viga)</t>
+          <t>6 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>5 (muro bajo la viga)</t>
+          <t>7 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -1134,8 +1134,16 @@
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n"/>
       <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
-      <c r="O10" s="2" t="n"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>2#4 -100/-75</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>2#4 -100/-75</t>
+        </is>
+      </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
           <t>E#3 @10</t>
@@ -1157,38 +1165,38 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>EJE-5 [S2]</t>
+          <t>EJE-11</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>5 (muro bajo la viga)</t>
+          <t>1 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>6 (muro bajo la viga)</t>
+          <t>2 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1.72</v>
+        <v>1.83</v>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>15x60</t>
+          <t>15x80</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>3#8</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>3#8</t>
         </is>
       </c>
       <c r="J11" s="2" t="n"/>
@@ -1218,54 +1226,54 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>EJE-5 [S2]</t>
+          <t>EJE-11</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>6 (muro bajo la viga)</t>
+          <t>2 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>7 (muro bajo la viga)</t>
+          <t>3 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1.83</v>
+        <v>1.82</v>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>15x60</t>
+          <t>15x80</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>3#8</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="n"/>
+          <t>3#8</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2#8 260/60</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>2#8 260/60</t>
+        </is>
+      </c>
       <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>2#4 -100/-75</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>2#4 -100/-75</t>
-        </is>
-      </c>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="inlineStr">
         <is>
           <t>E#3 @10</t>
@@ -1291,20 +1299,20 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>1 (muro bajo la viga)</t>
+          <t>3 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>2 (muro bajo la viga)</t>
+          <t>4 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1.83</v>
+        <v>1.82</v>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
@@ -1352,20 +1360,20 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>2 (muro bajo la viga)</t>
+          <t>4 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>3 (muro bajo la viga)</t>
+          <t>5 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1.82</v>
+        <v>1.84</v>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
@@ -1382,18 +1390,18 @@
           <t>3#8</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>2#8 260/60</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>2#8 260/60</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2#8 280/60</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>2#8 280/60</t>
+        </is>
+      </c>
       <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="inlineStr">
@@ -1421,20 +1429,20 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>3 (muro bajo la viga)</t>
+          <t>5 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>4 (muro bajo la viga)</t>
+          <t>6 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1.82</v>
+        <v>1.83</v>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
@@ -1452,9 +1460,17 @@
         </is>
       </c>
       <c r="J15" s="2" t="n"/>
-      <c r="K15" s="2" t="n"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2#8 60/60</t>
+        </is>
+      </c>
       <c r="L15" s="2" t="n"/>
-      <c r="M15" s="2" t="n"/>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>2#8 60/60</t>
+        </is>
+      </c>
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="n"/>
       <c r="P15" s="2" t="inlineStr">
@@ -1482,20 +1498,20 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>4 (muro bajo la viga)</t>
+          <t>6 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>5 (muro bajo la viga)</t>
+          <t>7 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1.84</v>
+        <v>1.83</v>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
@@ -1513,17 +1529,9 @@
         </is>
       </c>
       <c r="J16" s="2" t="n"/>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>2#8 280/60</t>
-        </is>
-      </c>
+      <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>2#8 280/60</t>
-        </is>
-      </c>
+      <c r="M16" s="2" t="n"/>
       <c r="N16" s="2" t="n"/>
       <c r="O16" s="2" t="n"/>
       <c r="P16" s="2" t="inlineStr">
@@ -1551,20 +1559,20 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>5 (muro bajo la viga)</t>
+          <t>7 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>6 (muro bajo la viga)</t>
+          <t>8 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1.83</v>
+        <v>1.63</v>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
@@ -1582,17 +1590,9 @@
         </is>
       </c>
       <c r="J17" s="2" t="n"/>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2#8 60/60</t>
-        </is>
-      </c>
+      <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>2#8 60/60</t>
-        </is>
-      </c>
+      <c r="M17" s="2" t="n"/>
       <c r="N17" s="2" t="n"/>
       <c r="O17" s="2" t="n"/>
       <c r="P17" s="2" t="inlineStr">
@@ -1620,20 +1620,20 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>6 (muro bajo la viga)</t>
+          <t>8 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>7 (muro bajo la viga)</t>
+          <t>9 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1.83</v>
+        <v>1.63</v>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
@@ -1654,8 +1654,16 @@
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
       <c r="M18" s="2" t="n"/>
-      <c r="N18" s="2" t="n"/>
-      <c r="O18" s="2" t="n"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>2#6 -100/-100</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2#6 -100/-100</t>
+        </is>
+      </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
           <t>E#3 @10</t>
@@ -1681,20 +1689,20 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>7 (muro bajo la viga)</t>
+          <t>9 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>8 (muro bajo la viga)</t>
+          <t>10 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1.63</v>
+        <v>1.82</v>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
@@ -1712,9 +1720,17 @@
         </is>
       </c>
       <c r="J19" s="2" t="n"/>
-      <c r="K19" s="2" t="n"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>2#6 60/250</t>
+        </is>
+      </c>
       <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="n"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>2#6 60/250</t>
+        </is>
+      </c>
       <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="inlineStr">
@@ -1742,20 +1758,20 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>8 (muro bajo la viga)</t>
+          <t>10 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>9 (muro bajo la viga)</t>
+          <t>11 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1.63</v>
+        <v>1.83</v>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
@@ -1776,16 +1792,8 @@
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n"/>
       <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>2#6 -100/-100</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>2#6 -100/-100</t>
-        </is>
-      </c>
+      <c r="N20" s="2" t="n"/>
+      <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="inlineStr">
         <is>
           <t>E#3 @10</t>
@@ -1807,52 +1815,48 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>EJE-11</t>
+          <t>T-5 (viga 2) [S1, S2]</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>9 (muro bajo la viga)</t>
+          <t>1 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>10 (muro bajo la viga)</t>
+          <t>2 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1.82</v>
+        <v>1.83</v>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>15x80</t>
+          <t>15x60</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>3#8</t>
+          <t>2#6</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>3#8</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>2#6 60/250</t>
+          <t>3#6 400/120</t>
         </is>
       </c>
       <c r="L21" s="2" t="n"/>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>2#6 60/250</t>
-        </is>
-      </c>
+      <c r="M21" s="2" t="n"/>
       <c r="N21" s="2" t="n"/>
       <c r="O21" s="2" t="n"/>
       <c r="P21" s="2" t="inlineStr">
@@ -1866,7 +1870,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S21" s="2" t="n"/>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas: ejes 5-8 (S1+S2) y ejes 9-11 (S3, 30X80); cada parte se arma aparte. | Plano: ejes 5-8 (sup. 2#6, inf. 3#6, bastón sup. 3#6 del extremo a 120 cm pasando el muro) y ejes 9-11 (30X80, 3#12). Los tramos 5 y 6 (30x80 antes del eje 9) no vienen detallados: se supuso 3#12 @10. | secciones: T-5 Seccion 1 + T-5 Seccion 2 + T-5 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1876,38 +1884,38 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>EJE-11</t>
+          <t>T-5 (viga 2) [S1, S2]</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>10 (muro bajo la viga)</t>
+          <t>2 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>11 (muro bajo la viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1.83</v>
+        <v>0.01</v>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>15x80</t>
+          <t>15x40</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>3#8</t>
+          <t>2#6</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>3#8</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="J22" s="2" t="n"/>
@@ -1918,7 +1926,7 @@
       <c r="O22" s="2" t="n"/>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>E#3 @10</t>
+          <t>E#3 @20</t>
         </is>
       </c>
       <c r="Q22" s="2" t="n"/>
@@ -1941,24 +1949,24 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>1 (muro bajo la viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>2 (muro bajo la viga)</t>
+          <t>4 (viga)</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1.83</v>
+        <v>1.51</v>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>15x60</t>
+          <t>15x40</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1972,18 +1980,14 @@
         </is>
       </c>
       <c r="J23" s="2" t="n"/>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>3#6 400/120</t>
-        </is>
-      </c>
+      <c r="K23" s="2" t="n"/>
       <c r="L23" s="2" t="n"/>
       <c r="M23" s="2" t="n"/>
       <c r="N23" s="2" t="n"/>
       <c r="O23" s="2" t="n"/>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>E#3 @10</t>
+          <t>E#3 11@10 @20 -</t>
         </is>
       </c>
       <c r="Q23" s="2" t="n"/>
@@ -1992,11 +1996,7 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S23" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas: ejes 5-8 (S1+S2) y ejes 9-11 (S3, 30X80); cada parte se arma aparte. | Plano: ejes 5-8 (sup. 2#6, inf. 3#6, bastón sup. 3#6 del extremo a 120 cm pasando el muro) y ejes 9-11 (30X80, 3#12). Los tramos 5 y 6 (30x80 antes del eje 9) no vienen detallados: se supuso 3#12 @10. | secciones: T-5 Seccion 1 + T-5 Seccion 2 + T-5 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
-        </is>
-      </c>
+      <c r="S23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2010,20 +2010,20 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>2 (muro bajo la viga)</t>
+          <t>4 (viga)</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>5 (viga)</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.01</v>
+        <v>1.66</v>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>E#3 @20</t>
+          <t>E#3 - @20 11@10</t>
         </is>
       </c>
       <c r="Q24" s="2" t="n"/>
@@ -2067,38 +2067,38 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2) [S1, S2]</t>
+          <t>T-5 (viga 2) [S3]</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1.51</v>
+        <v>6.12</v>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>15x40</t>
+          <t>30x80</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2#6</t>
+          <t>3#12</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>3#6</t>
+          <t>3#12</t>
         </is>
       </c>
       <c r="J25" s="2" t="n"/>
@@ -2106,10 +2106,14 @@
       <c r="L25" s="2" t="n"/>
       <c r="M25" s="2" t="n"/>
       <c r="N25" s="2" t="n"/>
-      <c r="O25" s="2" t="n"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>3#12 80</t>
+        </is>
+      </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>E#3 11@10 @20 -</t>
+          <t>E#3 11@10 @20 11@10</t>
         </is>
       </c>
       <c r="Q25" s="2" t="n"/>
@@ -2118,7 +2122,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S25" s="2" t="n"/>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas: ejes 5-8 (S1+S2) y ejes 9-11 (S3, 30X80); cada parte se arma aparte.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2128,33 +2136,33 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2) [S1, S2]</t>
+          <t>T-6 (viga 2) [S2]</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>5 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1.66</v>
+        <v>8.82</v>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>15x40</t>
+          <t>30x80</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2#6</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2167,10 +2175,14 @@
       <c r="L26" s="2" t="n"/>
       <c r="M26" s="2" t="n"/>
       <c r="N26" s="2" t="n"/>
-      <c r="O26" s="2" t="n"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>2#6 130</t>
+        </is>
+      </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>E#3 - @20 11@10</t>
+          <t>E#3 11@10,5@15 @20</t>
         </is>
       </c>
       <c r="Q26" s="2" t="n"/>
@@ -2179,7 +2191,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S26" s="2" t="n"/>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas: 30X80 (S2) y 15X80 (S3); cada parte se arma aparte. | Los tramos 2 y 3 (30x80 entre ejes 8 y 9) no vienen detallados: se supuso @10. | secciones: T-6 Seccion 2 + T-6 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2189,7 +2205,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2) [S3]</t>
+          <t>T-6 (viga 2) [S3]</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -2202,36 +2218,40 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>CS1 (cambio de sección)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.5</v>
+        <v>2.56</v>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>30x80</t>
+          <t>15x80</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>3#12</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>3#12</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="J27" s="2" t="n"/>
-      <c r="K27" s="2" t="n"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>2#6 90/120</t>
+        </is>
+      </c>
       <c r="L27" s="2" t="n"/>
       <c r="M27" s="2" t="n"/>
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>E#3 @10</t>
+          <t>E#3 11@10 @20 11@10</t>
         </is>
       </c>
       <c r="Q27" s="2" t="n"/>
@@ -2242,7 +2262,7 @@
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>En el plano son vigas separadas: ejes 5-8 (S1+S2) y ejes 9-11 (S3, 30X80); cada parte se arma aparte.</t>
+          <t>En el plano son vigas separadas: 30X80 (S2) y 15X80 (S3); cada parte se arma aparte.</t>
         </is>
       </c>
     </row>
@@ -2254,7 +2274,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2) [S3]</t>
+          <t>T-6 (viga 2) [S3]</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -2262,30 +2282,30 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>CS1 (cambio de sección)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>2 (viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.5</v>
+        <v>3.41</v>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>30x80</t>
+          <t>15x80</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>3#12</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>3#12</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="J28" s="2" t="n"/>
@@ -2296,7 +2316,7 @@
       <c r="O28" s="2" t="n"/>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>E#3 @10</t>
+          <t>E#3 11@10 @20 11@10</t>
         </is>
       </c>
       <c r="Q28" s="2" t="n"/>
@@ -2306,392 +2326,6 @@
         </is>
       </c>
       <c r="S28" s="2" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Nivel Roof Garden</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>T-5 (viga 2) [S3]</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>3</v>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>3 (viga)</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>6.12</v>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>30x80</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>3#12</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>3#12</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="n"/>
-      <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="n"/>
-      <c r="M29" s="2" t="n"/>
-      <c r="N29" s="2" t="n"/>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>3#12 80</t>
-        </is>
-      </c>
-      <c r="P29" s="2" t="inlineStr">
-        <is>
-          <t>E#3 11@10 @20 11@10</t>
-        </is>
-      </c>
-      <c r="Q29" s="2" t="n"/>
-      <c r="R29" s="2" t="inlineStr">
-        <is>
-          <t>#3@30</t>
-        </is>
-      </c>
-      <c r="S29" s="2" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Nivel Roof Garden</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>T-6 (viga 2) [S2]</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>1 (viga)</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>8.82</v>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>30x80</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="n"/>
-      <c r="K30" s="2" t="n"/>
-      <c r="L30" s="2" t="n"/>
-      <c r="M30" s="2" t="n"/>
-      <c r="N30" s="2" t="n"/>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>2#6 130</t>
-        </is>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>E#3 11@10,5@15 @20</t>
-        </is>
-      </c>
-      <c r="Q30" s="2" t="n"/>
-      <c r="R30" s="2" t="inlineStr">
-        <is>
-          <t>#3@30</t>
-        </is>
-      </c>
-      <c r="S30" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas: 30X80 (S2) y 15X80 (S3); cada parte se arma aparte. | Los tramos 2 y 3 (30x80 entre ejes 8 y 9) no vienen detallados: se supuso @10. | secciones: T-6 Seccion 2 + T-6 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Nivel Roof Garden</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>T-6 (viga 2) [S2]</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>2</v>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>CS1 (cambio de sección)</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>30x80</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="n"/>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="n"/>
-      <c r="N31" s="2" t="n"/>
-      <c r="O31" s="2" t="n"/>
-      <c r="P31" s="2" t="inlineStr">
-        <is>
-          <t>E#3 @10</t>
-        </is>
-      </c>
-      <c r="Q31" s="2" t="n"/>
-      <c r="R31" s="2" t="inlineStr">
-        <is>
-          <t>#3@30</t>
-        </is>
-      </c>
-      <c r="S31" s="2" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Nivel Roof Garden</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>T-6 (viga 2) [S2]</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>3</v>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>CS1 (cambio de sección)</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>3 (viga)</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>30x80</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="n"/>
-      <c r="K32" s="2" t="n"/>
-      <c r="L32" s="2" t="n"/>
-      <c r="M32" s="2" t="n"/>
-      <c r="N32" s="2" t="n"/>
-      <c r="O32" s="2" t="n"/>
-      <c r="P32" s="2" t="inlineStr">
-        <is>
-          <t>E#3 @10</t>
-        </is>
-      </c>
-      <c r="Q32" s="2" t="n"/>
-      <c r="R32" s="2" t="inlineStr">
-        <is>
-          <t>#3@30</t>
-        </is>
-      </c>
-      <c r="S32" s="2" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Nivel Roof Garden</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>T-6 (viga 2) [S3]</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>1 (viga)</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>2.56</v>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>15x80</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="n"/>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>2#6 90/120</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="n"/>
-      <c r="M33" s="2" t="n"/>
-      <c r="N33" s="2" t="n"/>
-      <c r="O33" s="2" t="n"/>
-      <c r="P33" s="2" t="inlineStr">
-        <is>
-          <t>E#3 11@10 @20 11@10</t>
-        </is>
-      </c>
-      <c r="Q33" s="2" t="n"/>
-      <c r="R33" s="2" t="inlineStr">
-        <is>
-          <t>#3@30</t>
-        </is>
-      </c>
-      <c r="S33" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas: 30X80 (S2) y 15X80 (S3); cada parte se arma aparte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Nivel Roof Garden</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>T-6 (viga 2) [S3]</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>2</v>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>3 (viga)</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>3.41</v>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>15x80</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="n"/>
-      <c r="K34" s="2" t="n"/>
-      <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="n"/>
-      <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="n"/>
-      <c r="P34" s="2" t="inlineStr">
-        <is>
-          <t>E#3 11@10 @20 11@10</t>
-        </is>
-      </c>
-      <c r="Q34" s="2" t="n"/>
-      <c r="R34" s="2" t="inlineStr">
-        <is>
-          <t>#3@30</t>
-        </is>
-      </c>
-      <c r="S34" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:S247"/>

</xml_diff>

<commit_message>
Insurgentes SD: drop gap spans without a beam element (T-2, T-2', T-6, EJE-J)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mu9wxeehZ5MxBaqNG8frbT
</commit_message>
<xml_diff>
--- a/revit/ArmadoTrabes_Insurgentes/Correccion_Roof_Garden_N10.xlsx
+++ b/revit/ArmadoTrabes_Insurgentes/Correccion_Roof_Garden_N10.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S40"/>
+  <dimension ref="A1:S35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>EJE-J [T1-2]</t>
+          <t>EJE-J [T1]</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>En el plano son vigas separadas: ejes 3-8 (2#6) y ejes 8-10 (3#4); cada parte se arma aparte.</t>
+          <t>En el plano son vigas separadas: ejes 3-8 (2#6) y ejes 8-10 (3#4). Entre el muro y la viga que cruza no hay trabe en el modelo (hueco del plano).</t>
         </is>
       </c>
     </row>
@@ -1230,24 +1230,24 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>EJE-J [T1-2]</t>
+          <t>EJE-J [T3]</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2 (muro bajo la viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>2.56</v>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
@@ -1256,12 +1256,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2#6</t>
+          <t>3#4</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2#6</t>
+          <t>3#4</t>
         </is>
       </c>
       <c r="J12" s="2" t="n"/>
@@ -1272,7 +1272,7 @@
       <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>E#3 @10</t>
+          <t>E#3 11@10 @20 11@10</t>
         </is>
       </c>
       <c r="Q12" s="2" t="n"/>
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>EJE-J [T3]</t>
+          <t>T-2 (viga 1) [T1-2]</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1308,11 +1308,11 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.56</v>
+        <v>1.01</v>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>15x60</t>
+          <t>15x40</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1333,7 +1333,7 @@
       <c r="O13" s="2" t="n"/>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>E#3 11@10 @20 11@10</t>
+          <t>E#3 11@10 @20 -</t>
         </is>
       </c>
       <c r="Q13" s="2" t="n"/>
@@ -1342,7 +1342,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S13" s="2" t="n"/>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos); entre los dos cajones no hay trabe en el modelo (hueco del plano): cada cajón se arma aparte.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1356,20 +1360,20 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>1 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>2 (viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1.01</v>
+        <v>1.4</v>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
@@ -1394,7 +1398,7 @@
       <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>E#3 11@10 @20 -</t>
+          <t>E#3 - @20 11@10</t>
         </is>
       </c>
       <c r="Q14" s="2" t="n"/>
@@ -1403,11 +1407,7 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S14" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado. | 4 vigas separadas con esta trabe: cada una con sus filas (el paréntesis dice los ejes de sus extremos)</t>
-        </is>
-      </c>
+      <c r="S14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1417,20 +1417,20 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 1) [T1-2]</t>
+          <t>T-2 (viga 1) [T4-5]</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
+          <t>1 (viga)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
           <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1459,7 +1459,7 @@
       <c r="O15" s="2" t="n"/>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>E#3 - @20 11@10</t>
+          <t>E#3 11@10 @20 -</t>
         </is>
       </c>
       <c r="Q15" s="2" t="n"/>
@@ -1468,7 +1468,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S15" s="2" t="n"/>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1478,24 +1482,24 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 1) [T3]</t>
+          <t>T-2 (viga 1) [T4-5]</t>
         </is>
       </c>
       <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>2 (viga)</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>3 (viga)</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
         <v>1</v>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>1 (viga)</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="F16" t="n">
-        <v>1.03</v>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
@@ -1520,7 +1524,7 @@
       <c r="O16" s="2" t="n"/>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>E#3 11@10 @20 11@10</t>
+          <t>E#3 - @20 11@10</t>
         </is>
       </c>
       <c r="Q16" s="2" t="n"/>
@@ -1529,11 +1533,7 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S16" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
-        </is>
-      </c>
+      <c r="S16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 1) [T4-5]</t>
+          <t>T-2 (viga 2) [T1-2]</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1.4</v>
+        <v>1.01</v>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+          <t>En el plano son vigas separadas (cajones distintos); entre los dos cajones no hay trabe en el modelo (hueco del plano): cada cajón se arma aparte.</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 1) [T4-5]</t>
+          <t>T-2 (viga 2) [T1-2]</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1625,7 +1625,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2) [T1-2]</t>
+          <t>T-2 (viga 2) [T4-6]</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1.01</v>
+        <v>0.72</v>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2) [T1-2]</t>
+          <t>T-2 (viga 2) [T4-6]</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1.4</v>
+        <v>0.54</v>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
@@ -1776,7 +1776,7 @@
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>E#3 - @20 11@10</t>
+          <t>E#3 @20</t>
         </is>
       </c>
       <c r="Q20" s="2" t="n"/>
@@ -1795,24 +1795,24 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2) [T3]</t>
+          <t>T-2 (viga 2) [T4-6]</t>
         </is>
       </c>
       <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>3 (viga)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>4 (viga)</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
         <v>1</v>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>1 (viga)</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>1.03</v>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
       <c r="O21" s="2" t="n"/>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>E#3 11@10 @20 11@10</t>
+          <t>E#3 - @20 11@10</t>
         </is>
       </c>
       <c r="Q21" s="2" t="n"/>
@@ -1846,11 +1846,7 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S21" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
-        </is>
-      </c>
+      <c r="S21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1860,7 +1856,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2) [T4-6]</t>
+          <t>T-2' (viga 1) [T1-2]</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1877,7 +1873,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.72</v>
+        <v>1.01</v>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
@@ -1913,7 +1909,7 @@
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+          <t>En el plano son vigas separadas (cajones distintos); entre los dos cajones no hay trabe en el modelo (hueco del plano): cada cajón se arma aparte.</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1921,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2) [T4-6]</t>
+          <t>T-2' (viga 1) [T1-2]</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1942,7 +1938,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.54</v>
+        <v>1.39</v>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
@@ -1967,7 +1963,7 @@
       <c r="O23" s="2" t="n"/>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>E#3 @20</t>
+          <t>E#3 - @20 11@10</t>
         </is>
       </c>
       <c r="Q23" s="2" t="n"/>
@@ -1986,24 +1982,24 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>T-2 (viga 2) [T4-6]</t>
+          <t>T-2' (viga 1) [T4-5]</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
@@ -2028,7 +2024,7 @@
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>E#3 - @20 11@10</t>
+          <t>E#3 11@10 @20 -</t>
         </is>
       </c>
       <c r="Q24" s="2" t="n"/>
@@ -2037,7 +2033,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S24" s="2" t="n"/>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2047,24 +2047,24 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>T-2' (viga 1) [T1-2]</t>
+          <t>T-2' (viga 1) [T4-5]</t>
         </is>
       </c>
       <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>2 (viga)</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>3 (viga)</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
         <v>1</v>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>1 (viga)</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>1.01</v>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
@@ -2089,7 +2089,7 @@
       <c r="O25" s="2" t="n"/>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>E#3 11@10 @20 -</t>
+          <t>E#3 - @20 11@10</t>
         </is>
       </c>
       <c r="Q25" s="2" t="n"/>
@@ -2098,11 +2098,7 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S25" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado. | 2 vigas separadas con esta trabe: cada una con sus filas (el paréntesis dice los ejes de sus extremos)</t>
-        </is>
-      </c>
+      <c r="S25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2112,49 +2108,53 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>T-2' (viga 1) [T1-2]</t>
+          <t>T-5 (viga 2) [S1, S2]</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>2 (viga)</t>
+          <t>1 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>2 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1.39</v>
+        <v>1.83</v>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>15x40</t>
+          <t>15x60</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>2#6</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="J26" s="2" t="n"/>
-      <c r="K26" s="2" t="n"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>3#6 400/120</t>
+        </is>
+      </c>
       <c r="L26" s="2" t="n"/>
       <c r="M26" s="2" t="n"/>
       <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>E#3 - @20 11@10</t>
+          <t>E#3 @10</t>
         </is>
       </c>
       <c r="Q26" s="2" t="n"/>
@@ -2163,7 +2163,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S26" s="2" t="n"/>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas: ejes 5-8 (S1+S2) y ejes 9-11 (S3, 30X80); cada parte se arma aparte. | Plano: ejes 5-8 (sup. 2#6, inf. 3#6, bastón sup. 3#6 del extremo a 120 cm pasando el muro) y ejes 9-11 (30X80, 3#12). Los tramos 5 y 6 (30x80 antes del eje 9) no vienen detallados: se supuso 3#12 @10. | secciones: T-5 Seccion 1 + T-5 Seccion 2 + T-5 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2173,24 +2177,24 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>T-2' (viga 1) [T3]</t>
+          <t>T-5 (viga 2) [S1, S2]</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>1 (viga)</t>
+          <t>2 (muro bajo la viga)</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>2 (viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1.03</v>
+        <v>0.01</v>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
@@ -2199,12 +2203,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>2#6</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="J27" s="2" t="n"/>
@@ -2215,7 +2219,7 @@
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>E#3 11@10 @20 11@10</t>
+          <t>E#3 @20</t>
         </is>
       </c>
       <c r="Q27" s="2" t="n"/>
@@ -2224,11 +2228,7 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S27" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
-        </is>
-      </c>
+      <c r="S27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2238,24 +2238,24 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>T-2' (viga 1) [T4-5]</t>
+          <t>T-5 (viga 2) [S1, S2]</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>1 (viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>2 (viga)</t>
+          <t>4 (viga)</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1.4</v>
+        <v>1.51</v>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
@@ -2264,12 +2264,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>2#6</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="J28" s="2" t="n"/>
@@ -2289,11 +2289,7 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S28" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
-        </is>
-      </c>
+      <c r="S28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2303,24 +2299,24 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>T-2' (viga 1) [T4-5]</t>
+          <t>T-5 (viga 2) [S1, S2]</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>2 (viga)</t>
+          <t>4 (viga)</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>5 (viga)</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>1.66</v>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
@@ -2329,12 +2325,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>2#6</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="J29" s="2" t="n"/>
@@ -2364,7 +2360,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2) [S1, S2]</t>
+          <t>T-5 (viga 2) [S3]</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -2372,45 +2368,45 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>1 (muro bajo la viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>2 (muro bajo la viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1.83</v>
+        <v>6.12</v>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>15x60</t>
+          <t>30x80</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2#6</t>
+          <t>3#12</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>3#6</t>
+          <t>3#12</t>
         </is>
       </c>
       <c r="J30" s="2" t="n"/>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>3#6 400/120</t>
-        </is>
-      </c>
+      <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="n"/>
       <c r="M30" s="2" t="n"/>
       <c r="N30" s="2" t="n"/>
-      <c r="O30" s="2" t="n"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>3#12 80</t>
+        </is>
+      </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>E#3 @10</t>
+          <t>E#3 11@10 @20 11@10</t>
         </is>
       </c>
       <c r="Q30" s="2" t="n"/>
@@ -2421,7 +2417,7 @@
       </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>En el plano son vigas separadas: ejes 5-8 (S1+S2) y ejes 9-11 (S3, 30X80); cada parte se arma aparte. | Plano: ejes 5-8 (sup. 2#6, inf. 3#6, bastón sup. 3#6 del extremo a 120 cm pasando el muro) y ejes 9-11 (30X80, 3#12). Los tramos 5 y 6 (30x80 antes del eje 9) no vienen detallados: se supuso 3#12 @10. | secciones: T-5 Seccion 1 + T-5 Seccion 2 + T-5 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
+          <t>En el plano son vigas separadas: ejes 5-8 (S1+S2) y ejes 9-11 (S3, 30X80); cada parte se arma aparte.</t>
         </is>
       </c>
     </row>
@@ -2433,38 +2429,38 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2) [S1, S2]</t>
+          <t>T-6 (viga 1) [T1]</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>2 (muro bajo la viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.01</v>
+        <v>2.56</v>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>15x40</t>
+          <t>15x60</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>2#6</t>
+          <t>3#4</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>3#6</t>
+          <t>3#4</t>
         </is>
       </c>
       <c r="J31" s="2" t="n"/>
@@ -2475,7 +2471,7 @@
       <c r="O31" s="2" t="n"/>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>E#3 @20</t>
+          <t>E#3 11@10 @20 11@10</t>
         </is>
       </c>
       <c r="Q31" s="2" t="n"/>
@@ -2484,7 +2480,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S31" s="2" t="n"/>
+      <c r="S31" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos); entre los dos cajones no hay trabe en el modelo (hueco del plano): cada cajón se arma aparte.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2494,38 +2494,38 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2) [S1, S2]</t>
+          <t>T-6 (viga 1) [T3]</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>3 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>2 (muro)</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1.51</v>
+        <v>2.55</v>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>15x40</t>
+          <t>15x60</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>2#6</t>
+          <t>3#4</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>3#6</t>
+          <t>3#4</t>
         </is>
       </c>
       <c r="J32" s="2" t="n"/>
@@ -2536,7 +2536,7 @@
       <c r="O32" s="2" t="n"/>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>E#3 11@10 @20 -</t>
+          <t>E#3 11@10 @20 11@10</t>
         </is>
       </c>
       <c r="Q32" s="2" t="n"/>
@@ -2545,7 +2545,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S32" s="2" t="n"/>
+      <c r="S32" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2555,33 +2559,33 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2) [S1, S2]</t>
+          <t>T-6 (viga 2) [S2]</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>4 (viga)</t>
+          <t>1 (viga)</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>5 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1.66</v>
+        <v>8.82</v>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>15x40</t>
+          <t>30x80</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>2#6</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2594,10 +2598,14 @@
       <c r="L33" s="2" t="n"/>
       <c r="M33" s="2" t="n"/>
       <c r="N33" s="2" t="n"/>
-      <c r="O33" s="2" t="n"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>2#6 130</t>
+        </is>
+      </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>E#3 - @20 11@10</t>
+          <t>E#3 11@10,5@15 @20</t>
         </is>
       </c>
       <c r="Q33" s="2" t="n"/>
@@ -2606,7 +2614,11 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S33" s="2" t="n"/>
+      <c r="S33" s="2" t="inlineStr">
+        <is>
+          <t>En el plano son vigas separadas: 30X80 (S2) y 15X80 (S3); cada parte se arma aparte. | Los tramos 2 y 3 (30x80 entre ejes 8 y 9) no vienen detallados: se supuso @10. | secciones: T-6 Seccion 2 + T-6 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2616,7 +2628,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>T-5 (viga 2) [S3]</t>
+          <t>T-6 (viga 2) [S3]</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -2633,33 +2645,33 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>6.12</v>
+        <v>2.56</v>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>30x80</t>
+          <t>15x80</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>3#12</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>3#12</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="J34" s="2" t="n"/>
-      <c r="K34" s="2" t="n"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>2#6 90/120</t>
+        </is>
+      </c>
       <c r="L34" s="2" t="n"/>
       <c r="M34" s="2" t="n"/>
       <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="inlineStr">
-        <is>
-          <t>3#12 80</t>
-        </is>
-      </c>
+      <c r="O34" s="2" t="n"/>
       <c r="P34" s="2" t="inlineStr">
         <is>
           <t>E#3 11@10 @20 11@10</t>
@@ -2673,7 +2685,7 @@
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>En el plano son vigas separadas: ejes 5-8 (S1+S2) y ejes 9-11 (S3, 30X80); cada parte se arma aparte.</t>
+          <t>En el plano son vigas separadas: 30X80 (S2) y 15X80 (S3); cada parte se arma aparte.</t>
         </is>
       </c>
     </row>
@@ -2685,38 +2697,38 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>T-6 (viga 1) [T1]</t>
+          <t>T-6 (viga 2) [S3]</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>1 (viga)</t>
+          <t>2 (viga)</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>2 (viga)</t>
+          <t>3 (viga)</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.56</v>
+        <v>3.41</v>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>15x60</t>
+          <t>15x80</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>3#4</t>
+          <t>3#6</t>
         </is>
       </c>
       <c r="J35" s="2" t="n"/>
@@ -2736,340 +2748,7 @@
           <t>#3@30</t>
         </is>
       </c>
-      <c r="S35" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado. | 2 vigas separadas con esta trabe: cada una con sus filas (el paréntesis dice los ejes de sus extremos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Nivel Roof Garden</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>T-6 (viga 1) [T2]</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>1 (viga)</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>15x60</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>3#4</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>3#4</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="n"/>
-      <c r="K36" s="2" t="n"/>
-      <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="n"/>
-      <c r="N36" s="2" t="n"/>
-      <c r="O36" s="2" t="n"/>
-      <c r="P36" s="2" t="inlineStr">
-        <is>
-          <t>E#3 11@10 @20 11@10</t>
-        </is>
-      </c>
-      <c r="Q36" s="2" t="n"/>
-      <c r="R36" s="2" t="inlineStr">
-        <is>
-          <t>#3@30</t>
-        </is>
-      </c>
-      <c r="S36" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Nivel Roof Garden</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>T-6 (viga 1) [T3]</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>1 (viga)</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>2 (muro)</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>15x60</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>3#4</t>
-        </is>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>3#4</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="n"/>
-      <c r="K37" s="2" t="n"/>
-      <c r="L37" s="2" t="n"/>
-      <c r="M37" s="2" t="n"/>
-      <c r="N37" s="2" t="n"/>
-      <c r="O37" s="2" t="n"/>
-      <c r="P37" s="2" t="inlineStr">
-        <is>
-          <t>E#3 11@10 @20 11@10</t>
-        </is>
-      </c>
-      <c r="Q37" s="2" t="n"/>
-      <c r="R37" s="2" t="inlineStr">
-        <is>
-          <t>#3@30</t>
-        </is>
-      </c>
-      <c r="S37" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas (cajones distintos): cada parte se arma aparte. El tramo entre los dos cajones no viene en el plano: se supuso el mismo armado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Nivel Roof Garden</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>T-6 (viga 2) [S2]</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>1 (viga)</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>8.82</v>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>30x80</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="n"/>
-      <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="n"/>
-      <c r="M38" s="2" t="n"/>
-      <c r="N38" s="2" t="n"/>
-      <c r="O38" s="2" t="inlineStr">
-        <is>
-          <t>2#6 130</t>
-        </is>
-      </c>
-      <c r="P38" s="2" t="inlineStr">
-        <is>
-          <t>E#3 11@10,5@15 @20</t>
-        </is>
-      </c>
-      <c r="Q38" s="2" t="n"/>
-      <c r="R38" s="2" t="inlineStr">
-        <is>
-          <t>#3@30</t>
-        </is>
-      </c>
-      <c r="S38" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas: 30X80 (S2) y 15X80 (S3); cada parte se arma aparte. | Los tramos 2 y 3 (30x80 entre ejes 8 y 9) no vienen detallados: se supuso @10. | secciones: T-6 Seccion 2 + T-6 Seccion 3 (se arman juntas; los bastones pasan el cambio de sección)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Nivel Roof Garden</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>T-6 (viga 2) [S3]</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>1 (viga)</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>2.56</v>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>15x80</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="n"/>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>2#6 90/120</t>
-        </is>
-      </c>
-      <c r="L39" s="2" t="n"/>
-      <c r="M39" s="2" t="n"/>
-      <c r="N39" s="2" t="n"/>
-      <c r="O39" s="2" t="n"/>
-      <c r="P39" s="2" t="inlineStr">
-        <is>
-          <t>E#3 11@10 @20 11@10</t>
-        </is>
-      </c>
-      <c r="Q39" s="2" t="n"/>
-      <c r="R39" s="2" t="inlineStr">
-        <is>
-          <t>#3@30</t>
-        </is>
-      </c>
-      <c r="S39" s="2" t="inlineStr">
-        <is>
-          <t>En el plano son vigas separadas: 30X80 (S2) y 15X80 (S3); cada parte se arma aparte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Nivel Roof Garden</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>T-6 (viga 2) [S3]</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>2</v>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>2 (viga)</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>3 (viga)</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>3.41</v>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>15x80</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>3#6</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="n"/>
-      <c r="K40" s="2" t="n"/>
-      <c r="L40" s="2" t="n"/>
-      <c r="M40" s="2" t="n"/>
-      <c r="N40" s="2" t="n"/>
-      <c r="O40" s="2" t="n"/>
-      <c r="P40" s="2" t="inlineStr">
-        <is>
-          <t>E#3 11@10 @20 11@10</t>
-        </is>
-      </c>
-      <c r="Q40" s="2" t="n"/>
-      <c r="R40" s="2" t="inlineStr">
-        <is>
-          <t>#3@30</t>
-        </is>
-      </c>
-      <c r="S40" s="2" t="n"/>
+      <c r="S35" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:S247"/>

</xml_diff>